<commit_message>
Module 3 completed - steps 1-8
</commit_message>
<xml_diff>
--- a/week-09/NorthwindTablesAndColumns.xlsx
+++ b/week-09/NorthwindTablesAndColumns.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nataliamiranda\Documents\DataAnalytics\week-09\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D5A05F1-2E49-40AC-8232-ADDCCC840D47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFEB0F30-1634-426C-AEDC-3AF6BB64A693}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{901F5D27-877F-4C94-89AE-9A9B6ECE5CB6}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{901F5D27-877F-4C94-89AE-9A9B6ECE5CB6}"/>
   </bookViews>
   <sheets>
     <sheet name="Northwind Columns" sheetId="1" r:id="rId1"/>
@@ -352,12 +352,6 @@
     <t>Employee Photo</t>
   </si>
   <si>
-    <t>Customer Company Name</t>
-  </si>
-  <si>
-    <t>Customer Contact Name</t>
-  </si>
-  <si>
     <t>Customer Contact Title</t>
   </si>
   <si>
@@ -391,9 +385,6 @@
     <t>Shippers Company Name</t>
   </si>
   <si>
-    <t>Supplier Company Name</t>
-  </si>
-  <si>
     <t>Supplier Contact Name</t>
   </si>
   <si>
@@ -926,6 +917,15 @@
   </si>
   <si>
     <t xml:space="preserve">Primary key; needed for relationship to Products </t>
+  </si>
+  <si>
+    <t>Customer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer Contact </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supplier </t>
   </si>
 </sst>
 </file>
@@ -1528,19 +1528,19 @@
         <v>95</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="N2" s="18" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="31" x14ac:dyDescent="0.35">
@@ -1572,19 +1572,19 @@
         <v>100</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="N3" s="18" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="46.5" x14ac:dyDescent="0.35">
@@ -1616,19 +1616,19 @@
         <v>101</v>
       </c>
       <c r="J4" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="L4" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="K4" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="L4" s="8" t="s">
-        <v>173</v>
-      </c>
       <c r="M4" s="8" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="N4" s="18" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="31" x14ac:dyDescent="0.35">
@@ -1660,19 +1660,19 @@
         <v>102</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K5" s="8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L5" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="M5" s="8" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="N5" s="18" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="46.5" x14ac:dyDescent="0.35">
@@ -1704,19 +1704,19 @@
         <v>96</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L6" s="9" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="M6" s="9" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="31" x14ac:dyDescent="0.35">
@@ -1745,22 +1745,22 @@
         <v>93</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>105</v>
+        <v>294</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L7" s="9" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M7" s="9" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="31" x14ac:dyDescent="0.35">
@@ -1789,22 +1789,22 @@
         <v>93</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>106</v>
+        <v>295</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L8" s="9" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M8" s="9" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="31" x14ac:dyDescent="0.35">
@@ -1833,22 +1833,22 @@
         <v>93</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K9" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L9" s="9" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M9" s="9" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="N9" s="7" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="46.5" x14ac:dyDescent="0.35">
@@ -1877,22 +1877,22 @@
         <v>94</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K10" s="9" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L10" s="9" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M10" s="9" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="N10" s="7" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="31" x14ac:dyDescent="0.35">
@@ -1921,25 +1921,25 @@
         <v>93</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K11" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L11" s="9" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="M11" s="9" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="N11" s="7" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" s="15" t="s">
         <v>16</v>
       </c>
@@ -1965,25 +1965,25 @@
         <v>93</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L12" s="9" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="M12" s="9" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="N12" s="7" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" ht="46.5" x14ac:dyDescent="0.35">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="31" x14ac:dyDescent="0.35">
       <c r="A13" s="15" t="s">
         <v>16</v>
       </c>
@@ -2009,25 +2009,25 @@
         <v>93</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K13" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L13" s="9" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="M13" s="9" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="N13" s="7" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" s="15" t="s">
         <v>16</v>
       </c>
@@ -2053,25 +2053,25 @@
         <v>93</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L14" s="9" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="M14" s="9" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="N14" s="7" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" s="15" t="s">
         <v>16</v>
       </c>
@@ -2097,25 +2097,25 @@
         <v>94</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L15" s="9" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M15" s="9" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="N15" s="7" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" s="15" t="s">
         <v>16</v>
       </c>
@@ -2141,25 +2141,25 @@
         <v>94</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K16" s="9" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L16" s="9" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M16" s="9" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="N16" s="7" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" ht="46.5" x14ac:dyDescent="0.35">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" ht="31" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>27</v>
       </c>
@@ -2188,22 +2188,22 @@
         <v>97</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K17" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L17" s="8" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="M17" s="8" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="N17" s="18" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>27</v>
       </c>
@@ -2229,25 +2229,25 @@
         <v>93</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K18" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L18" s="8" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M18" s="8" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="N18" s="18" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
         <v>27</v>
       </c>
@@ -2273,25 +2273,25 @@
         <v>93</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K19" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L19" s="8" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M19" s="8" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="N19" s="18" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
         <v>27</v>
       </c>
@@ -2317,25 +2317,25 @@
         <v>93</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K20" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L20" s="8" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M20" s="8" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="N20" s="18" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>27</v>
       </c>
@@ -2361,25 +2361,25 @@
         <v>94</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K21" s="8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L21" s="8" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M21" s="8" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="N21" s="18" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>27</v>
       </c>
@@ -2405,25 +2405,25 @@
         <v>93</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K22" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L22" s="8" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="M22" s="8" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="N22" s="18" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="23" spans="1:14" ht="46.5" x14ac:dyDescent="0.35">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
         <v>27</v>
       </c>
@@ -2449,25 +2449,25 @@
         <v>93</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K23" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L23" s="8" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="M23" s="8" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="N23" s="18" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
         <v>27</v>
       </c>
@@ -2496,22 +2496,22 @@
         <v>103</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K24" s="8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L24" s="8" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M24" s="8" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="N24" s="18" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
         <v>27</v>
       </c>
@@ -2537,25 +2537,25 @@
         <v>93</v>
       </c>
       <c r="I25" s="5" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="J25" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K25" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L25" s="8" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="M25" s="8" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="N25" s="18" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="26" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
         <v>27</v>
       </c>
@@ -2581,25 +2581,25 @@
         <v>93</v>
       </c>
       <c r="I26" s="5" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K26" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L26" s="8" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="M26" s="8" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="N26" s="18" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>27</v>
       </c>
@@ -2625,25 +2625,25 @@
         <v>93</v>
       </c>
       <c r="I27" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="J27" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K27" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L27" s="8" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="M27" s="8" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="N27" s="18" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="28" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
         <v>27</v>
       </c>
@@ -2669,25 +2669,25 @@
         <v>93</v>
       </c>
       <c r="I28" s="5" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="J28" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K28" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L28" s="8" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="M28" s="8" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="N28" s="18" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="29" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
         <v>27</v>
       </c>
@@ -2713,25 +2713,25 @@
         <v>94</v>
       </c>
       <c r="I29" s="5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J29" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K29" s="8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L29" s="8" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M29" s="8" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="N29" s="18" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="30" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
         <v>27</v>
       </c>
@@ -2757,25 +2757,25 @@
         <v>94</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K30" s="8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L30" s="8" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M30" s="8" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="N30" s="18" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="31" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
         <v>27</v>
       </c>
@@ -2804,22 +2804,22 @@
         <v>104</v>
       </c>
       <c r="J31" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K31" s="8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L31" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="M31" s="8" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="N31" s="18" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="32" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
         <v>27</v>
       </c>
@@ -2845,25 +2845,25 @@
         <v>94</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="J32" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="K32" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="L32" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="K32" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="L32" s="8" t="s">
-        <v>173</v>
-      </c>
       <c r="M32" s="8" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="N32" s="18" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="33" spans="1:14" ht="46.5" x14ac:dyDescent="0.35">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" ht="31" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
         <v>27</v>
       </c>
@@ -2889,25 +2889,25 @@
         <v>93</v>
       </c>
       <c r="I33" s="5" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="J33" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K33" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L33" s="8" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="M33" s="8" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="N33" s="18" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="34" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
         <v>27</v>
       </c>
@@ -2933,25 +2933,25 @@
         <v>94</v>
       </c>
       <c r="I34" s="5" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J34" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K34" s="8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L34" s="8" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="M34" s="8" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="N34" s="18" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="35" spans="1:14" ht="62" x14ac:dyDescent="0.35">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" ht="31" x14ac:dyDescent="0.35">
       <c r="A35" s="15" t="s">
         <v>42</v>
       </c>
@@ -2980,22 +2980,22 @@
         <v>97</v>
       </c>
       <c r="J35" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K35" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L35" s="9" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="M35" s="9" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="N35" s="7" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="36" spans="1:14" ht="46.5" x14ac:dyDescent="0.35">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" ht="31" x14ac:dyDescent="0.35">
       <c r="A36" s="15" t="s">
         <v>42</v>
       </c>
@@ -3024,22 +3024,22 @@
         <v>98</v>
       </c>
       <c r="J36" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K36" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L36" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="M36" s="9" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="N36" s="7" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="37" spans="1:14" ht="46.5" x14ac:dyDescent="0.35">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" ht="31" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
         <v>44</v>
       </c>
@@ -3065,25 +3065,25 @@
         <v>93</v>
       </c>
       <c r="I37" s="5" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="J37" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K37" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L37" s="8" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="M37" s="8" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="N37" s="18" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="38" spans="1:14" ht="46.5" x14ac:dyDescent="0.35">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" ht="31" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
         <v>44</v>
       </c>
@@ -3109,25 +3109,25 @@
         <v>93</v>
       </c>
       <c r="I38" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="J38" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K38" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L38" s="8" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="M38" s="8" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="N38" s="18" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="39" spans="1:14" ht="46.5" x14ac:dyDescent="0.35">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" ht="31" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
         <v>44</v>
       </c>
@@ -3153,25 +3153,25 @@
         <v>93</v>
       </c>
       <c r="I39" s="5" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="J39" s="5" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="K39" s="8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L39" s="8" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="M39" s="8" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="N39" s="18" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="40" spans="1:14" ht="46.5" x14ac:dyDescent="0.35">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="31" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
         <v>44</v>
       </c>
@@ -3197,25 +3197,25 @@
         <v>93</v>
       </c>
       <c r="I40" s="5" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="J40" s="5" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="K40" s="8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L40" s="8" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="M40" s="8" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="N40" s="18" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="41" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
         <v>44</v>
       </c>
@@ -3241,25 +3241,25 @@
         <v>93</v>
       </c>
       <c r="I41" s="5" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="J41" s="5" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="K41" s="8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L41" s="8" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="M41" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="N41" s="18" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="42" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A42" s="11" t="s">
         <v>53</v>
       </c>
@@ -3285,25 +3285,25 @@
         <v>93</v>
       </c>
       <c r="I42" s="6" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="J42" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K42" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L42" s="9" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="M42" s="9" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="N42" s="7" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="43" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A43" s="11" t="s">
         <v>53</v>
       </c>
@@ -3332,22 +3332,22 @@
         <v>96</v>
       </c>
       <c r="J43" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K43" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L43" s="9" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="M43" s="9" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="N43" s="7" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="44" spans="1:14" ht="46.5" x14ac:dyDescent="0.35">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" ht="31" x14ac:dyDescent="0.35">
       <c r="A44" s="11" t="s">
         <v>53</v>
       </c>
@@ -3376,22 +3376,22 @@
         <v>97</v>
       </c>
       <c r="J44" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K44" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L44" s="9" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="M44" s="9" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="N44" s="7" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="45" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A45" s="11" t="s">
         <v>53</v>
       </c>
@@ -3417,25 +3417,25 @@
         <v>93</v>
       </c>
       <c r="I45" s="6" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K45" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L45" s="9" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="M45" s="9" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="N45" s="7" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="46" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A46" s="11" t="s">
         <v>53</v>
       </c>
@@ -3461,25 +3461,25 @@
         <v>93</v>
       </c>
       <c r="I46" s="6" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="J46" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K46" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L46" s="9" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="M46" s="9" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="N46" s="7" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="47" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A47" s="11" t="s">
         <v>53</v>
       </c>
@@ -3505,22 +3505,22 @@
         <v>93</v>
       </c>
       <c r="I47" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="J47" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K47" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L47" s="9" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="M47" s="9" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="N47" s="7" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
     </row>
     <row r="48" spans="1:14" ht="31" x14ac:dyDescent="0.35">
@@ -3549,25 +3549,25 @@
         <v>93</v>
       </c>
       <c r="I48" s="6" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="J48" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K48" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L48" s="9" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="M48" s="9" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="N48" s="7" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="49" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A49" s="11" t="s">
         <v>53</v>
       </c>
@@ -3593,25 +3593,25 @@
         <v>93</v>
       </c>
       <c r="I49" s="6" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="J49" s="16" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="K49" s="9" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L49" s="9" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="M49" s="9" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="N49" s="7" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="50" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A50" s="11" t="s">
         <v>53</v>
       </c>
@@ -3637,25 +3637,25 @@
         <v>93</v>
       </c>
       <c r="I50" s="6" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="J50" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K50" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L50" s="9" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M50" s="9" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="N50" s="7" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="51" spans="1:14" ht="46.5" x14ac:dyDescent="0.35">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" ht="31" x14ac:dyDescent="0.35">
       <c r="A51" s="11" t="s">
         <v>53</v>
       </c>
@@ -3681,25 +3681,25 @@
         <v>94</v>
       </c>
       <c r="I51" s="6" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="J51" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K51" s="9" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L51" s="9" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M51" s="9" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="N51" s="7" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="52" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A52" s="11" t="s">
         <v>53</v>
       </c>
@@ -3725,25 +3725,25 @@
         <v>93</v>
       </c>
       <c r="I52" s="6" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="J52" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K52" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L52" s="9" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="M52" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="N52" s="7" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="53" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A53" s="11" t="s">
         <v>53</v>
       </c>
@@ -3769,25 +3769,25 @@
         <v>93</v>
       </c>
       <c r="I53" s="6" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="J53" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K53" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L53" s="9" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="M53" s="9" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="N53" s="7" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="54" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A54" s="11" t="s">
         <v>53</v>
       </c>
@@ -3813,25 +3813,25 @@
         <v>93</v>
       </c>
       <c r="I54" s="6" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="J54" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K54" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L54" s="9" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="M54" s="9" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="N54" s="7" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="55" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A55" s="11" t="s">
         <v>53</v>
       </c>
@@ -3857,25 +3857,25 @@
         <v>93</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="J55" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K55" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L55" s="9" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="M55" s="9" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="N55" s="7" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="56" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
         <v>65</v>
       </c>
@@ -3901,22 +3901,22 @@
         <v>93</v>
       </c>
       <c r="I56" s="5" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="J56" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K56" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L56" s="8" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="M56" s="8" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="N56" s="18" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="57" spans="1:14" ht="31" x14ac:dyDescent="0.35">
@@ -3945,22 +3945,22 @@
         <v>93</v>
       </c>
       <c r="I57" s="5" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="J57" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K57" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L57" s="8" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M57" s="8" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="N57" s="18" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
     </row>
     <row r="58" spans="1:14" ht="31" x14ac:dyDescent="0.35">
@@ -3989,22 +3989,22 @@
         <v>93</v>
       </c>
       <c r="I58" s="5" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="J58" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K58" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L58" s="8" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="M58" s="8" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="N58" s="18" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="59" spans="1:14" ht="31" x14ac:dyDescent="0.35">
@@ -4036,22 +4036,22 @@
         <v>95</v>
       </c>
       <c r="J59" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K59" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L59" s="8" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="M59" s="8" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="N59" s="18" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="60" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A60" s="3" t="s">
         <v>65</v>
       </c>
@@ -4077,22 +4077,22 @@
         <v>93</v>
       </c>
       <c r="I60" s="5" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="J60" s="5" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="K60" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L60" s="8" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M60" s="8" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="N60" s="18" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
     </row>
     <row r="61" spans="1:14" ht="31" x14ac:dyDescent="0.35">
@@ -4121,25 +4121,25 @@
         <v>93</v>
       </c>
       <c r="I61" s="5" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="J61" s="5" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="K61" s="8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L61" s="8" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="M61" s="8" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="N61" s="18" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="62" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
         <v>65</v>
       </c>
@@ -4165,25 +4165,25 @@
         <v>93</v>
       </c>
       <c r="I62" s="5" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="J62" s="5" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="K62" s="8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L62" s="8" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="M62" s="8" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="N62" s="18" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="63" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A63" s="3" t="s">
         <v>65</v>
       </c>
@@ -4209,25 +4209,25 @@
         <v>93</v>
       </c>
       <c r="I63" s="5" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J63" s="5" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="K63" s="8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L63" s="8" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="M63" s="8" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="N63" s="18" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="64" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A64" s="3" t="s">
         <v>65</v>
       </c>
@@ -4253,25 +4253,25 @@
         <v>93</v>
       </c>
       <c r="I64" s="5" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="J64" s="5" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="K64" s="8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L64" s="8" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="M64" s="8" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="N64" s="18" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="65" spans="1:14" ht="46.5" x14ac:dyDescent="0.35">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="65" spans="1:14" ht="31" x14ac:dyDescent="0.35">
       <c r="A65" s="3" t="s">
         <v>65</v>
       </c>
@@ -4300,22 +4300,22 @@
         <v>72</v>
       </c>
       <c r="J65" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K65" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L65" s="8" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="M65" s="8" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="N65" s="18" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="66" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A66" s="11" t="s">
         <v>22</v>
       </c>
@@ -4344,22 +4344,22 @@
         <v>99</v>
       </c>
       <c r="J66" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K66" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L66" s="9" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="M66" s="9" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="N66" s="7" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="67" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A67" s="11" t="s">
         <v>22</v>
       </c>
@@ -4385,25 +4385,25 @@
         <v>94</v>
       </c>
       <c r="I67" s="6" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="J67" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K67" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L67" s="9" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M67" s="9" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="N67" s="7" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="68" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A68" s="3" t="s">
         <v>76</v>
       </c>
@@ -4429,25 +4429,25 @@
         <v>93</v>
       </c>
       <c r="I68" s="5" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="J68" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K68" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L68" s="8" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="M68" s="8" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="N68" s="18" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="69" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A69" s="3" t="s">
         <v>76</v>
       </c>
@@ -4473,25 +4473,25 @@
         <v>93</v>
       </c>
       <c r="I69" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="J69" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K69" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L69" s="8" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M69" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="N69" s="18" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="70" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A70" s="3" t="s">
         <v>76</v>
       </c>
@@ -4517,25 +4517,25 @@
         <v>94</v>
       </c>
       <c r="I70" s="5" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="J70" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K70" s="8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L70" s="8" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M70" s="8" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="N70" s="18" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="71" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A71" s="11" t="s">
         <v>78</v>
       </c>
@@ -4561,25 +4561,25 @@
         <v>93</v>
       </c>
       <c r="I71" s="6" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="J71" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K71" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L71" s="9" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="M71" s="9" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="N71" s="7" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="72" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A72" s="11" t="s">
         <v>78</v>
       </c>
@@ -4605,25 +4605,25 @@
         <v>93</v>
       </c>
       <c r="I72" s="6" t="s">
-        <v>118</v>
+        <v>296</v>
       </c>
       <c r="J72" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K72" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L72" s="9" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M72" s="9" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="N72" s="7" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="73" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A73" s="11" t="s">
         <v>78</v>
       </c>
@@ -4649,25 +4649,25 @@
         <v>93</v>
       </c>
       <c r="I73" s="6" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="J73" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K73" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L73" s="9" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M73" s="9" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="N73" s="7" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="74" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A74" s="11" t="s">
         <v>78</v>
       </c>
@@ -4693,25 +4693,25 @@
         <v>93</v>
       </c>
       <c r="I74" s="6" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="J74" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K74" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L74" s="9" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M74" s="9" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="N74" s="7" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="75" spans="1:14" ht="46.5" x14ac:dyDescent="0.35">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14" ht="31" x14ac:dyDescent="0.35">
       <c r="A75" s="11" t="s">
         <v>78</v>
       </c>
@@ -4737,25 +4737,25 @@
         <v>94</v>
       </c>
       <c r="I75" s="6" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="J75" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K75" s="9" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L75" s="9" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M75" s="9" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="N75" s="7" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="76" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A76" s="11" t="s">
         <v>78</v>
       </c>
@@ -4781,25 +4781,25 @@
         <v>93</v>
       </c>
       <c r="I76" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="J76" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K76" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L76" s="9" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="M76" s="9" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="N76" s="7" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="77" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A77" s="11" t="s">
         <v>78</v>
       </c>
@@ -4825,25 +4825,25 @@
         <v>93</v>
       </c>
       <c r="I77" s="6" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J77" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K77" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L77" s="9" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="M77" s="9" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="N77" s="7" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="78" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A78" s="11" t="s">
         <v>78</v>
       </c>
@@ -4869,22 +4869,22 @@
         <v>93</v>
       </c>
       <c r="I78" s="6" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="J78" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K78" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L78" s="9" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="M78" s="9" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="N78" s="7" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="79" spans="1:14" ht="31" x14ac:dyDescent="0.35">
@@ -4913,25 +4913,25 @@
         <v>93</v>
       </c>
       <c r="I79" s="6" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="J79" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K79" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L79" s="9" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="M79" s="9" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="N79" s="7" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="80" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A80" s="11" t="s">
         <v>78</v>
       </c>
@@ -4957,25 +4957,25 @@
         <v>94</v>
       </c>
       <c r="I80" s="6" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="J80" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K80" s="9" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L80" s="9" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M80" s="9" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="N80" s="7" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="81" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="81" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A81" s="11" t="s">
         <v>78</v>
       </c>
@@ -5001,25 +5001,25 @@
         <v>94</v>
       </c>
       <c r="I81" s="6" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="J81" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K81" s="9" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L81" s="9" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M81" s="9" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="N81" s="7" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="82" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A82" s="11" t="s">
         <v>78</v>
       </c>
@@ -5045,25 +5045,25 @@
         <v>94</v>
       </c>
       <c r="I82" s="6" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="J82" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K82" s="9" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L82" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="M82" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="M82" s="9" t="s">
-        <v>191</v>
-      </c>
       <c r="N82" s="7" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="83" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A83" s="3" t="s">
         <v>80</v>
       </c>
@@ -5089,25 +5089,25 @@
         <v>93</v>
       </c>
       <c r="I83" s="5" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="J83" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K83" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L83" s="8" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="M83" s="8" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="N83" s="18" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="84" spans="1:14" ht="31" x14ac:dyDescent="0.35">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="84" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A84" s="3" t="s">
         <v>80</v>
       </c>
@@ -5133,22 +5133,22 @@
         <v>94</v>
       </c>
       <c r="I84" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="J84" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="K84" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="L84" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="J84" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="K84" s="8" t="s">
-        <v>171</v>
-      </c>
-      <c r="L84" s="8" t="s">
-        <v>172</v>
-      </c>
       <c r="M84" s="8" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="N84" s="18" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="85" spans="1:14" ht="31" x14ac:dyDescent="0.35">
@@ -5180,19 +5180,19 @@
         <v>99</v>
       </c>
       <c r="J85" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K85" s="14" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L85" s="14" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="M85" s="14" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="N85" s="19" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
     </row>
     <row r="86" spans="1:14" x14ac:dyDescent="0.35">
@@ -5205,6 +5205,34 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="ced60a7f-99b1-48d2-b555-34851c8026ae" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9e0b35a9-e6cb-436b-81d4-4440ba439ca5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <SharedWithUsers xmlns="ced60a7f-99b1-48d2-b555-34851c8026ae">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <MediaLengthInSeconds xmlns="9e0b35a9-e6cb-436b-81d4-4440ba439ca5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CA5D0A6329BB324E86983B32928CFC2E" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3d7eac4bce3bbb09c82bd908806be82e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9e0b35a9-e6cb-436b-81d4-4440ba439ca5" xmlns:ns3="ced60a7f-99b1-48d2-b555-34851c8026ae" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eb51570e5b7cb8bd524bc2df5324d4a3" ns2:_="" ns3:_="">
     <xsd:import namespace="9e0b35a9-e6cb-436b-81d4-4440ba439ca5"/>
@@ -5445,35 +5473,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="ced60a7f-99b1-48d2-b555-34851c8026ae" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9e0b35a9-e6cb-436b-81d4-4440ba439ca5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <SharedWithUsers xmlns="ced60a7f-99b1-48d2-b555-34851c8026ae">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <MediaLengthInSeconds xmlns="9e0b35a9-e6cb-436b-81d4-4440ba439ca5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0257D61C-6042-483B-9C34-3DE0D82CB154}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BB560F9-4CC1-4243-8F16-7FDC2CD703FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ced60a7f-99b1-48d2-b555-34851c8026ae"/>
+    <ds:schemaRef ds:uri="9e0b35a9-e6cb-436b-81d4-4440ba439ca5"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA285021-94D7-4152-B2E7-B2D9504C2DBD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5490,23 +5509,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BB560F9-4CC1-4243-8F16-7FDC2CD703FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ced60a7f-99b1-48d2-b555-34851c8026ae"/>
-    <ds:schemaRef ds:uri="9e0b35a9-e6cb-436b-81d4-4440ba439ca5"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0257D61C-6042-483B-9C34-3DE0D82CB154}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>